<commit_message>
Full integration of caching feature [Final Commit?]
- integrated aengl5337's data caching feature preventing downloading new
  data if up to date data already exists.

- build_exe.py now copies the DATA folder alongside wb_list.xlsx into
  the distribution folder, so cached FAA/DCS/flight/fuel/comment data
  ships with the exe (stale data is auto-refreshed on first run via
  Alec's CycleCache cycle-date comparison)

- minor bug fixes.
</commit_message>
<xml_diff>
--- a/wb_list.xlsx
+++ b/wb_list.xlsx
@@ -862,12 +862,12 @@
       </c>
       <c r="Q2" s="19" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="R2" s="19" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CJO</t>
         </is>
       </c>
       <c r="S2" s="19" t="inlineStr">
@@ -949,17 +949,17 @@
       </c>
       <c r="Q3" s="19" t="inlineStr">
         <is>
-          <t>2026-01-29</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="R3" s="19" t="inlineStr">
         <is>
-          <t>JWG</t>
+          <t>CJO</t>
         </is>
       </c>
       <c r="S3" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="T3" s="19" t="n"/>
@@ -1017,17 +1017,17 @@
       </c>
       <c r="Q4" s="19" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="R4" s="19" t="inlineStr">
         <is>
+          <t>CJO</t>
+        </is>
+      </c>
+      <c r="S4" s="19" t="inlineStr">
+        <is>
           <t>CMC</t>
-        </is>
-      </c>
-      <c r="S4" s="19" t="inlineStr">
-        <is>
-          <t>PRT</t>
         </is>
       </c>
       <c r="T4" s="19" t="n"/>
@@ -1085,17 +1085,17 @@
       </c>
       <c r="Q5" s="19" t="inlineStr">
         <is>
-          <t>2026-01-28</t>
+          <t>2026-02-05</t>
         </is>
       </c>
       <c r="R5" s="19" t="inlineStr">
         <is>
-          <t>CBI</t>
+          <t>AFU</t>
         </is>
       </c>
       <c r="S5" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
+          <t>BAP</t>
         </is>
       </c>
       <c r="T5" s="19" t="n"/>
@@ -1153,16 +1153,18 @@
       </c>
       <c r="Q6" s="19" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R6" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
-        </is>
-      </c>
-      <c r="S6" s="19" t="n">
-        <v/>
+          <t>HAS</t>
+        </is>
+      </c>
+      <c r="S6" s="19" t="inlineStr">
+        <is>
+          <t>WSM</t>
+        </is>
       </c>
       <c r="T6" s="19" t="n"/>
       <c r="U6" s="19" t="inlineStr">
@@ -1220,17 +1222,17 @@
       </c>
       <c r="Q7" s="19" t="inlineStr">
         <is>
-          <t>2026-01-21</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R7" s="19" t="inlineStr">
         <is>
-          <t>JPJ</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="S7" s="19" t="inlineStr">
         <is>
-          <t>WLS</t>
+          <t>WSM</t>
         </is>
       </c>
       <c r="T7" s="19" t="n"/>
@@ -1289,17 +1291,17 @@
       </c>
       <c r="Q8" s="19" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R8" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>DDC</t>
         </is>
       </c>
       <c r="S8" s="19" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>JWA</t>
         </is>
       </c>
       <c r="T8" s="19" t="n"/>
@@ -1353,18 +1355,16 @@
       </c>
       <c r="Q9" s="19" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R9" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="S9" s="19" t="inlineStr">
-        <is>
-          <t>JAM</t>
-        </is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="S9" s="19" t="n">
+        <v/>
       </c>
       <c r="T9" s="19" t="n"/>
       <c r="U9" s="19" t="n"/>
@@ -1414,18 +1414,16 @@
       </c>
       <c r="Q10" s="19" t="inlineStr">
         <is>
-          <t>2026-01-18</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R10" s="19" t="inlineStr">
         <is>
-          <t>ADO</t>
-        </is>
-      </c>
-      <c r="S10" s="19" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="S10" s="19" t="n">
+        <v/>
       </c>
       <c r="T10" s="19" t="n"/>
       <c r="U10" s="19" t="n"/>
@@ -1471,17 +1469,17 @@
       </c>
       <c r="Q11" s="19" t="inlineStr">
         <is>
-          <t>2026-01-15</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R11" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>DDC</t>
         </is>
       </c>
       <c r="S11" s="19" t="inlineStr">
         <is>
-          <t>LOV</t>
+          <t>RBL</t>
         </is>
       </c>
       <c r="T11" s="19" t="n"/>
@@ -1529,17 +1527,17 @@
       </c>
       <c r="Q12" s="19" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="R12" s="19" t="inlineStr">
         <is>
-          <t>BAM</t>
+          <t>DDC</t>
         </is>
       </c>
       <c r="S12" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>RBL</t>
         </is>
       </c>
       <c r="T12" s="19" t="n"/>
@@ -1591,17 +1589,17 @@
       </c>
       <c r="Q13" s="19" t="inlineStr">
         <is>
-          <t>2026-01-13</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="R13" s="19" t="inlineStr">
         <is>
-          <t>KCO</t>
+          <t>CBI</t>
         </is>
       </c>
       <c r="S13" s="19" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>LDE</t>
         </is>
       </c>
       <c r="T13" s="19" t="n"/>
@@ -1648,17 +1646,17 @@
       </c>
       <c r="Q14" s="19" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="R14" s="19" t="inlineStr">
         <is>
-          <t>ADO</t>
+          <t>JWG</t>
         </is>
       </c>
       <c r="S14" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="T14" s="19" t="n"/>
@@ -1701,17 +1699,17 @@
       </c>
       <c r="Q15" s="19" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-28</t>
         </is>
       </c>
       <c r="R15" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="S15" s="19" t="inlineStr">
         <is>
-          <t>VAN</t>
+          <t>PRT</t>
         </is>
       </c>
       <c r="T15" s="19" t="n"/>
@@ -1754,18 +1752,16 @@
       </c>
       <c r="Q16" s="19" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="R16" s="19" t="inlineStr">
         <is>
-          <t>JWA</t>
-        </is>
-      </c>
-      <c r="S16" s="19" t="inlineStr">
-        <is>
-          <t>MAN</t>
-        </is>
+          <t>AWP</t>
+        </is>
+      </c>
+      <c r="S16" s="19" t="n">
+        <v/>
       </c>
       <c r="T16" s="19" t="n"/>
       <c r="U16" s="19" t="n"/>
@@ -1808,17 +1804,17 @@
       </c>
       <c r="Q17" s="19" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="R17" s="19" t="inlineStr">
         <is>
-          <t>CBI</t>
+          <t>JPJ</t>
         </is>
       </c>
       <c r="S17" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>WLS</t>
         </is>
       </c>
       <c r="T17" s="19" t="n"/>
@@ -1866,17 +1862,17 @@
       </c>
       <c r="Q18" s="19" t="inlineStr">
         <is>
-          <t>2025-12-18</t>
+          <t>2026-01-18</t>
         </is>
       </c>
       <c r="R18" s="19" t="inlineStr">
         <is>
-          <t>CBI</t>
+          <t>HMK</t>
         </is>
       </c>
       <c r="S18" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>WSM</t>
         </is>
       </c>
       <c r="T18" s="19" t="n"/>
@@ -1919,17 +1915,17 @@
       </c>
       <c r="Q19" s="19" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="R19" s="19" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>ADO</t>
         </is>
       </c>
       <c r="S19" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="T19" s="19" t="n"/>
@@ -1972,17 +1968,17 @@
       </c>
       <c r="Q20" s="19" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="R20" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>BRS</t>
         </is>
       </c>
       <c r="S20" s="19" t="inlineStr">
         <is>
-          <t>HMK</t>
+          <t>VAN</t>
         </is>
       </c>
       <c r="T20" s="19" t="n"/>
@@ -2026,17 +2022,17 @@
       </c>
       <c r="Q21" s="19" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="R21" s="19" t="inlineStr">
         <is>
-          <t>JMO</t>
+          <t>JWA</t>
         </is>
       </c>
       <c r="S21" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="T21" s="19" t="n"/>
@@ -2084,17 +2080,17 @@
       </c>
       <c r="Q22" s="19" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="R22" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>CBI</t>
         </is>
       </c>
       <c r="S22" s="19" t="inlineStr">
         <is>
-          <t>JMO</t>
+          <t>LDE</t>
         </is>
       </c>
       <c r="T22" s="19" t="n"/>
@@ -2137,17 +2133,17 @@
       </c>
       <c r="Q23" s="19" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
+          <t>2025-12-18</t>
         </is>
       </c>
       <c r="R23" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>CBI</t>
         </is>
       </c>
       <c r="S23" s="19" t="inlineStr">
         <is>
-          <t>LOV</t>
+          <t>LDE</t>
         </is>
       </c>
       <c r="T23" s="19" t="n"/>
@@ -2191,7 +2187,7 @@
       </c>
       <c r="Q24" s="19" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="R24" s="19" t="inlineStr">
@@ -2201,7 +2197,7 @@
       </c>
       <c r="S24" s="19" t="inlineStr">
         <is>
-          <t>TIN</t>
+          <t>LDE</t>
         </is>
       </c>
       <c r="T24" s="19" t="n"/>
@@ -2249,17 +2245,17 @@
       </c>
       <c r="Q25" s="19" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="R25" s="19" t="inlineStr">
         <is>
-          <t>CBI</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S25" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>HMK</t>
         </is>
       </c>
       <c r="T25" s="19" t="n"/>
@@ -2302,16 +2298,18 @@
       </c>
       <c r="Q26" s="19" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-12-09</t>
         </is>
       </c>
       <c r="R26" s="19" t="inlineStr">
         <is>
-          <t>MAN</t>
-        </is>
-      </c>
-      <c r="S26" s="19" t="n">
-        <v/>
+          <t>JMO</t>
+        </is>
+      </c>
+      <c r="S26" s="19" t="inlineStr">
+        <is>
+          <t>RJC</t>
+        </is>
       </c>
       <c r="T26" s="19" t="n"/>
       <c r="U26" s="19" t="n"/>
@@ -2354,7 +2352,7 @@
       </c>
       <c r="Q27" s="19" t="inlineStr">
         <is>
-          <t>2025-11-19</t>
+          <t>2025-12-02</t>
         </is>
       </c>
       <c r="R27" s="19" t="inlineStr">
@@ -2364,7 +2362,7 @@
       </c>
       <c r="S27" s="19" t="inlineStr">
         <is>
-          <t>FRU</t>
+          <t>LOV</t>
         </is>
       </c>
       <c r="T27" s="19" t="n"/>
@@ -2408,17 +2406,17 @@
       </c>
       <c r="Q28" s="19" t="inlineStr">
         <is>
-          <t>2025-11-14</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="R28" s="19" t="inlineStr">
         <is>
-          <t>LAO</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="S28" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
+          <t>TIN</t>
         </is>
       </c>
       <c r="T28" s="19" t="n"/>
@@ -2462,17 +2460,17 @@
       </c>
       <c r="Q29" s="19" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="R29" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
+          <t>CBI</t>
         </is>
       </c>
       <c r="S29" s="19" t="inlineStr">
         <is>
-          <t>LOV</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="T29" s="19" t="n"/>
@@ -2516,12 +2514,12 @@
       </c>
       <c r="Q30" s="19" t="inlineStr">
         <is>
-          <t>2025-11-06</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="R30" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="S30" s="19" t="n">
@@ -2568,17 +2566,17 @@
       </c>
       <c r="Q31" s="19" t="inlineStr">
         <is>
-          <t>2025-11-05</t>
+          <t>2025-11-19</t>
         </is>
       </c>
       <c r="R31" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
+          <t>BRS</t>
         </is>
       </c>
       <c r="S31" s="19" t="inlineStr">
         <is>
-          <t>BNE</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="T31" s="19" t="n"/>
@@ -2610,17 +2608,17 @@
       </c>
       <c r="Q32" s="19" t="inlineStr">
         <is>
-          <t>2025-11-04</t>
+          <t>2025-11-14</t>
         </is>
       </c>
       <c r="R32" s="19" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>LAO</t>
         </is>
       </c>
       <c r="S32" s="19" t="inlineStr">
         <is>
-          <t>RTH</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="T32" s="19" t="n"/>
@@ -2652,16 +2650,18 @@
       </c>
       <c r="Q33" s="19" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-11-06</t>
         </is>
       </c>
       <c r="R33" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
-        </is>
-      </c>
-      <c r="S33" s="19" t="n">
-        <v/>
+          <t>AWP</t>
+        </is>
+      </c>
+      <c r="S33" s="19" t="inlineStr">
+        <is>
+          <t>LOV</t>
+        </is>
       </c>
       <c r="T33" s="19" t="n"/>
       <c r="U33" s="19" t="n"/>
@@ -2692,12 +2692,12 @@
       </c>
       <c r="Q34" s="19" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-11-06</t>
         </is>
       </c>
       <c r="R34" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S34" s="19" t="n">
@@ -2732,16 +2732,18 @@
       </c>
       <c r="Q35" s="19" t="inlineStr">
         <is>
-          <t>2025-10-26</t>
+          <t>2025-11-05</t>
         </is>
       </c>
       <c r="R35" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
-        </is>
-      </c>
-      <c r="S35" s="19" t="n">
-        <v/>
+          <t>AWP</t>
+        </is>
+      </c>
+      <c r="S35" s="19" t="inlineStr">
+        <is>
+          <t>BNE</t>
+        </is>
       </c>
       <c r="T35" s="19" t="n"/>
       <c r="U35" s="19" t="n"/>
@@ -2772,16 +2774,18 @@
       </c>
       <c r="Q36" s="19" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-11-04</t>
         </is>
       </c>
       <c r="R36" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="S36" s="19" t="n">
-        <v/>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="S36" s="19" t="inlineStr">
+        <is>
+          <t>RTH</t>
+        </is>
       </c>
       <c r="T36" s="19" t="n"/>
       <c r="U36" s="19" t="n"/>
@@ -2812,18 +2816,16 @@
       </c>
       <c r="Q37" s="19" t="inlineStr">
         <is>
-          <t>2025-10-13</t>
+          <t>2025-10-26</t>
         </is>
       </c>
       <c r="R37" s="19" t="inlineStr">
         <is>
-          <t>BAP</t>
-        </is>
-      </c>
-      <c r="S37" s="19" t="inlineStr">
-        <is>
-          <t>FRU</t>
-        </is>
+          <t>DDC</t>
+        </is>
+      </c>
+      <c r="S37" s="19" t="n">
+        <v/>
       </c>
       <c r="T37" s="19" t="n"/>
       <c r="U37" s="19" t="n"/>
@@ -2854,7 +2856,7 @@
       </c>
       <c r="Q38" s="19" t="inlineStr">
         <is>
-          <t>2025-10-07</t>
+          <t>2025-10-26</t>
         </is>
       </c>
       <c r="R38" s="19" t="inlineStr">
@@ -2862,10 +2864,8 @@
           <t>DDC</t>
         </is>
       </c>
-      <c r="S38" s="19" t="inlineStr">
-        <is>
-          <t>LOV</t>
-        </is>
+      <c r="S38" s="19" t="n">
+        <v/>
       </c>
       <c r="T38" s="19" t="n"/>
       <c r="U38" s="19" t="n"/>
@@ -2896,18 +2896,16 @@
       </c>
       <c r="Q39" s="19" t="inlineStr">
         <is>
-          <t>2025-10-03</t>
+          <t>2025-10-26</t>
         </is>
       </c>
       <c r="R39" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
-        </is>
-      </c>
-      <c r="S39" s="19" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
+          <t>DDC</t>
+        </is>
+      </c>
+      <c r="S39" s="19" t="n">
+        <v/>
       </c>
       <c r="T39" s="19" t="n"/>
       <c r="U39" s="19" t="n"/>
@@ -2938,18 +2936,16 @@
       </c>
       <c r="Q40" s="19" t="inlineStr">
         <is>
-          <t>2025-09-29</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="R40" s="19" t="inlineStr">
         <is>
-          <t>AML</t>
-        </is>
-      </c>
-      <c r="S40" s="19" t="inlineStr">
-        <is>
-          <t>SMB</t>
-        </is>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="S40" s="19" t="n">
+        <v/>
       </c>
       <c r="T40" s="19" t="n"/>
       <c r="U40" s="19" t="n"/>
@@ -2980,17 +2976,17 @@
       </c>
       <c r="Q41" s="19" t="inlineStr">
         <is>
-          <t>2025-09-26</t>
+          <t>2025-10-13</t>
         </is>
       </c>
       <c r="R41" s="19" t="inlineStr">
         <is>
-          <t>AML</t>
+          <t>BAP</t>
         </is>
       </c>
       <c r="S41" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>FRU</t>
         </is>
       </c>
       <c r="T41" s="19" t="n"/>
@@ -3022,16 +3018,18 @@
       </c>
       <c r="Q42" s="19" t="inlineStr">
         <is>
-          <t>2025-09-25</t>
+          <t>2025-10-03</t>
         </is>
       </c>
       <c r="R42" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
-        </is>
-      </c>
-      <c r="S42" s="19" t="n">
-        <v/>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="S42" s="19" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
       </c>
       <c r="T42" s="19" t="n"/>
       <c r="U42" s="19" t="n"/>
@@ -3062,17 +3060,17 @@
       </c>
       <c r="Q43" s="19" t="inlineStr">
         <is>
-          <t>2025-09-22</t>
+          <t>2025-09-29</t>
         </is>
       </c>
       <c r="R43" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>AML</t>
         </is>
       </c>
       <c r="S43" s="19" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="T43" s="19" t="n"/>
@@ -3104,17 +3102,17 @@
       </c>
       <c r="Q44" s="19" t="inlineStr">
         <is>
-          <t>2025-09-18</t>
+          <t>2025-09-26</t>
         </is>
       </c>
       <c r="R44" s="19" t="inlineStr">
         <is>
-          <t>PWF</t>
+          <t>AML</t>
         </is>
       </c>
       <c r="S44" s="19" t="inlineStr">
         <is>
-          <t>RTH</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="T44" s="19" t="n"/>
@@ -3146,18 +3144,16 @@
       </c>
       <c r="Q45" s="19" t="inlineStr">
         <is>
-          <t>2025-09-11</t>
+          <t>2025-09-25</t>
         </is>
       </c>
       <c r="R45" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
-        </is>
-      </c>
-      <c r="S45" s="19" t="inlineStr">
-        <is>
-          <t>TIN</t>
-        </is>
+          <t>RJC</t>
+        </is>
+      </c>
+      <c r="S45" s="19" t="n">
+        <v/>
       </c>
       <c r="T45" s="19" t="n"/>
       <c r="U45" s="19" t="n"/>
@@ -3188,17 +3184,17 @@
       </c>
       <c r="Q46" s="19" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
+          <t>2025-09-22</t>
         </is>
       </c>
       <c r="R46" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
+          <t>LDE</t>
         </is>
       </c>
       <c r="S46" s="19" t="inlineStr">
         <is>
-          <t>KCO</t>
+          <t>MBE</t>
         </is>
       </c>
       <c r="T46" s="19" t="n"/>
@@ -3230,17 +3226,17 @@
       </c>
       <c r="Q47" s="19" t="inlineStr">
         <is>
-          <t>2025-08-22</t>
+          <t>2025-09-18</t>
         </is>
       </c>
       <c r="R47" s="19" t="inlineStr">
         <is>
-          <t>JWA</t>
+          <t>PWF</t>
         </is>
       </c>
       <c r="S47" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>RTH</t>
         </is>
       </c>
       <c r="T47" s="19" t="n"/>
@@ -3272,16 +3268,18 @@
       </c>
       <c r="Q48" s="19" t="inlineStr">
         <is>
-          <t>2025-08-03</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="R48" s="19" t="inlineStr">
         <is>
-          <t>BAP</t>
-        </is>
-      </c>
-      <c r="S48" s="19" t="n">
-        <v/>
+          <t>MBE</t>
+        </is>
+      </c>
+      <c r="S48" s="19" t="inlineStr">
+        <is>
+          <t>RJC</t>
+        </is>
       </c>
       <c r="T48" s="19" t="n"/>
       <c r="U48" s="19" t="n"/>
@@ -3312,16 +3310,18 @@
       </c>
       <c r="Q49" s="19" t="inlineStr">
         <is>
-          <t>2025-08-02</t>
+          <t>2025-09-03</t>
         </is>
       </c>
       <c r="R49" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
-        </is>
-      </c>
-      <c r="S49" s="19" t="n">
-        <v/>
+          <t>AWP</t>
+        </is>
+      </c>
+      <c r="S49" s="19" t="inlineStr">
+        <is>
+          <t>KCO</t>
+        </is>
       </c>
       <c r="T49" s="19" t="n"/>
       <c r="U49" s="19" t="n"/>
@@ -3352,16 +3352,18 @@
       </c>
       <c r="Q50" s="19" t="inlineStr">
         <is>
-          <t>2025-08-02</t>
+          <t>2025-08-22</t>
         </is>
       </c>
       <c r="R50" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
-        </is>
-      </c>
-      <c r="S50" s="19" t="n">
-        <v/>
+          <t>JWA</t>
+        </is>
+      </c>
+      <c r="S50" s="19" t="inlineStr">
+        <is>
+          <t>LDE</t>
+        </is>
       </c>
       <c r="T50" s="19" t="n"/>
       <c r="U50" s="19" t="n"/>
@@ -3392,18 +3394,16 @@
       </c>
       <c r="Q51" s="19" t="inlineStr">
         <is>
-          <t>2025-07-10</t>
+          <t>2025-08-03</t>
         </is>
       </c>
       <c r="R51" s="19" t="inlineStr">
         <is>
-          <t>ADO</t>
-        </is>
-      </c>
-      <c r="S51" s="19" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
+          <t>BAP</t>
+        </is>
+      </c>
+      <c r="S51" s="19" t="n">
+        <v/>
       </c>
       <c r="T51" s="19" t="n"/>
       <c r="U51" s="19" t="n"/>
@@ -3434,12 +3434,12 @@
       </c>
       <c r="Q52" s="19" t="inlineStr">
         <is>
-          <t>2025-07-06</t>
+          <t>2025-08-02</t>
         </is>
       </c>
       <c r="R52" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="S52" s="19" t="n">
@@ -3474,12 +3474,12 @@
       </c>
       <c r="Q53" s="19" t="inlineStr">
         <is>
-          <t>2025-07-05</t>
+          <t>2025-08-02</t>
         </is>
       </c>
       <c r="R53" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="S53" s="19" t="n">
@@ -3514,17 +3514,17 @@
       </c>
       <c r="Q54" s="19" t="inlineStr">
         <is>
-          <t>2025-07-02</t>
+          <t>2025-07-10</t>
         </is>
       </c>
       <c r="R54" s="19" t="inlineStr">
         <is>
-          <t>HMK</t>
+          <t>ADO</t>
         </is>
       </c>
       <c r="S54" s="19" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="T54" s="19" t="n"/>
@@ -3556,18 +3556,16 @@
       </c>
       <c r="Q55" s="19" t="inlineStr">
         <is>
-          <t>2025-07-02</t>
+          <t>2025-07-06</t>
         </is>
       </c>
       <c r="R55" s="19" t="inlineStr">
         <is>
-          <t>HMK</t>
-        </is>
-      </c>
-      <c r="S55" s="19" t="inlineStr">
-        <is>
-          <t>MAN</t>
-        </is>
+          <t>DDC</t>
+        </is>
+      </c>
+      <c r="S55" s="19" t="n">
+        <v/>
       </c>
       <c r="T55" s="19" t="n"/>
       <c r="U55" s="19" t="n"/>
@@ -3598,18 +3596,16 @@
       </c>
       <c r="Q56" s="19" t="inlineStr">
         <is>
-          <t>2025-06-30</t>
+          <t>2025-07-05</t>
         </is>
       </c>
       <c r="R56" s="19" t="inlineStr">
         <is>
-          <t>CWI</t>
-        </is>
-      </c>
-      <c r="S56" s="19" t="inlineStr">
-        <is>
-          <t>SMB</t>
-        </is>
+          <t>DDC</t>
+        </is>
+      </c>
+      <c r="S56" s="19" t="n">
+        <v/>
       </c>
       <c r="T56" s="19" t="n"/>
       <c r="U56" s="19" t="n"/>
@@ -3640,16 +3636,18 @@
       </c>
       <c r="Q57" s="19" t="inlineStr">
         <is>
-          <t>2025-06-22</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="R57" s="19" t="inlineStr">
         <is>
-          <t>WSM</t>
-        </is>
-      </c>
-      <c r="S57" s="19" t="n">
-        <v/>
+          <t>HMK</t>
+        </is>
+      </c>
+      <c r="S57" s="19" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
       </c>
       <c r="T57" s="19" t="n"/>
       <c r="U57" s="19" t="n"/>
@@ -3680,17 +3678,17 @@
       </c>
       <c r="Q58" s="19" t="inlineStr">
         <is>
-          <t>2025-06-20</t>
+          <t>2025-07-02</t>
         </is>
       </c>
       <c r="R58" s="19" t="inlineStr">
         <is>
-          <t>JHA</t>
+          <t>HMK</t>
         </is>
       </c>
       <c r="S58" s="19" t="inlineStr">
         <is>
-          <t>MIR</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="T58" s="19" t="n"/>
@@ -3722,16 +3720,18 @@
       </c>
       <c r="Q59" s="19" t="inlineStr">
         <is>
-          <t>2025-06-15</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="R59" s="19" t="inlineStr">
         <is>
+          <t>CWI</t>
+        </is>
+      </c>
+      <c r="S59" s="19" t="inlineStr">
+        <is>
           <t>SMB</t>
         </is>
-      </c>
-      <c r="S59" s="19" t="n">
-        <v/>
       </c>
       <c r="T59" s="19" t="n"/>
       <c r="U59" s="19" t="n"/>
@@ -3762,12 +3762,12 @@
       </c>
       <c r="Q60" s="19" t="inlineStr">
         <is>
-          <t>2025-06-13</t>
+          <t>2025-06-22</t>
         </is>
       </c>
       <c r="R60" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>WSM</t>
         </is>
       </c>
       <c r="S60" s="19" t="n">
@@ -3802,17 +3802,17 @@
       </c>
       <c r="Q61" s="19" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-06-20</t>
         </is>
       </c>
       <c r="R61" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
+          <t>JHA</t>
         </is>
       </c>
       <c r="S61" s="19" t="inlineStr">
         <is>
-          <t>WLS</t>
+          <t>MIR</t>
         </is>
       </c>
       <c r="T61" s="19" t="n"/>
@@ -3844,18 +3844,16 @@
       </c>
       <c r="Q62" s="19" t="inlineStr">
         <is>
-          <t>2025-06-04</t>
+          <t>2025-06-15</t>
         </is>
       </c>
       <c r="R62" s="19" t="inlineStr">
         <is>
-          <t>MBE</t>
-        </is>
-      </c>
-      <c r="S62" s="19" t="inlineStr">
-        <is>
-          <t>RJC</t>
-        </is>
+          <t>SMB</t>
+        </is>
+      </c>
+      <c r="S62" s="19" t="n">
+        <v/>
       </c>
       <c r="T62" s="19" t="n"/>
       <c r="U62" s="19" t="n"/>
@@ -3886,7 +3884,7 @@
       </c>
       <c r="Q63" s="19" t="inlineStr">
         <is>
-          <t>2025-05-23</t>
+          <t>2025-06-13</t>
         </is>
       </c>
       <c r="R63" s="19" t="inlineStr">
@@ -3926,16 +3924,18 @@
       </c>
       <c r="Q64" s="19" t="inlineStr">
         <is>
-          <t>2025-05-21</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="R64" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
-        </is>
-      </c>
-      <c r="S64" s="19" t="n">
-        <v/>
+          <t>AWP</t>
+        </is>
+      </c>
+      <c r="S64" s="19" t="inlineStr">
+        <is>
+          <t>WLS</t>
+        </is>
       </c>
       <c r="T64" s="19" t="n"/>
       <c r="U64" s="19" t="n"/>
@@ -3966,16 +3966,18 @@
       </c>
       <c r="Q65" s="19" t="inlineStr">
         <is>
-          <t>2025-05-21</t>
+          <t>2025-06-04</t>
         </is>
       </c>
       <c r="R65" s="19" t="inlineStr">
         <is>
+          <t>MBE</t>
+        </is>
+      </c>
+      <c r="S65" s="19" t="inlineStr">
+        <is>
           <t>RJC</t>
         </is>
-      </c>
-      <c r="S65" s="19" t="n">
-        <v/>
       </c>
       <c r="T65" s="19" t="n"/>
       <c r="U65" s="19" t="n"/>
@@ -4006,16 +4008,18 @@
       </c>
       <c r="Q66" s="19" t="inlineStr">
         <is>
-          <t>2025-05-21</t>
+          <t>2025-05-23</t>
         </is>
       </c>
       <c r="R66" s="19" t="inlineStr">
         <is>
-          <t>MAN</t>
-        </is>
-      </c>
-      <c r="S66" s="19" t="n">
-        <v/>
+          <t>JWG</t>
+        </is>
+      </c>
+      <c r="S66" s="19" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
       </c>
       <c r="T66" s="19" t="n"/>
       <c r="U66" s="19" t="n"/>
@@ -4046,12 +4050,12 @@
       </c>
       <c r="Q67" s="19" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2025-05-21</t>
         </is>
       </c>
       <c r="R67" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="S67" s="19" t="n">
@@ -4086,12 +4090,12 @@
       </c>
       <c r="Q68" s="19" t="inlineStr">
         <is>
-          <t>2025-04-20</t>
+          <t>2025-05-21</t>
         </is>
       </c>
       <c r="R68" s="19" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="S68" s="19" t="n">
@@ -4126,12 +4130,12 @@
       </c>
       <c r="Q69" s="19" t="inlineStr">
         <is>
-          <t>2025-04-19</t>
+          <t>2025-05-21</t>
         </is>
       </c>
       <c r="R69" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="S69" s="19" t="n">
@@ -4166,7 +4170,7 @@
       </c>
       <c r="Q70" s="19" t="inlineStr">
         <is>
-          <t>2025-04-19</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="R70" s="19" t="inlineStr">
@@ -4206,12 +4210,12 @@
       </c>
       <c r="Q71" s="19" t="inlineStr">
         <is>
-          <t>2025-04-19</t>
+          <t>2025-04-20</t>
         </is>
       </c>
       <c r="R71" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>HAS</t>
         </is>
       </c>
       <c r="S71" s="19" t="n">
@@ -4246,12 +4250,12 @@
       </c>
       <c r="Q72" s="19" t="inlineStr">
         <is>
-          <t>2025-03-11</t>
+          <t>2025-04-19</t>
         </is>
       </c>
       <c r="R72" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S72" s="19" t="n">
@@ -4286,7 +4290,7 @@
       </c>
       <c r="Q73" s="19" t="inlineStr">
         <is>
-          <t>2024-11-21</t>
+          <t>2025-04-19</t>
         </is>
       </c>
       <c r="R73" s="19" t="inlineStr">
@@ -4326,7 +4330,7 @@
       </c>
       <c r="Q74" s="19" t="inlineStr">
         <is>
-          <t>2024-11-21</t>
+          <t>2025-04-19</t>
         </is>
       </c>
       <c r="R74" s="19" t="inlineStr">
@@ -4366,12 +4370,12 @@
       </c>
       <c r="Q75" s="19" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="R75" s="19" t="inlineStr">
         <is>
-          <t>BRS</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="S75" s="19" t="n">
@@ -4406,18 +4410,16 @@
       </c>
       <c r="Q76" s="19" t="inlineStr">
         <is>
-          <t>2024-11-07</t>
+          <t>2024-11-21</t>
         </is>
       </c>
       <c r="R76" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
-        </is>
-      </c>
-      <c r="S76" s="19" t="inlineStr">
-        <is>
-          <t>JAM</t>
-        </is>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="S76" s="19" t="n">
+        <v/>
       </c>
       <c r="T76" s="19" t="n"/>
       <c r="U76" s="19" t="n"/>
@@ -4448,7 +4450,7 @@
       </c>
       <c r="Q77" s="19" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-11-21</t>
         </is>
       </c>
       <c r="R77" s="19" t="inlineStr">
@@ -4488,18 +4490,16 @@
       </c>
       <c r="Q78" s="19" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="R78" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="S78" s="19" t="inlineStr">
-        <is>
-          <t>WLS</t>
-        </is>
+          <t>BRS</t>
+        </is>
+      </c>
+      <c r="S78" s="19" t="n">
+        <v/>
       </c>
       <c r="T78" s="19" t="n"/>
       <c r="U78" s="19" t="n"/>
@@ -4530,17 +4530,17 @@
       </c>
       <c r="Q79" s="19" t="inlineStr">
         <is>
-          <t>2024-11-01</t>
+          <t>2024-11-07</t>
         </is>
       </c>
       <c r="R79" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>AWP</t>
         </is>
       </c>
       <c r="S79" s="19" t="inlineStr">
         <is>
-          <t>WLS</t>
+          <t>JAM</t>
         </is>
       </c>
       <c r="T79" s="19" t="n"/>
@@ -4572,7 +4572,7 @@
       </c>
       <c r="Q80" s="19" t="inlineStr">
         <is>
-          <t>2024-10-21</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="R80" s="19" t="inlineStr">
@@ -4580,10 +4580,8 @@
           <t>GLO</t>
         </is>
       </c>
-      <c r="S80" s="19" t="inlineStr">
-        <is>
-          <t>JHA</t>
-        </is>
+      <c r="S80" s="19" t="n">
+        <v/>
       </c>
       <c r="T80" s="19" t="n"/>
       <c r="U80" s="19" t="n"/>
@@ -4614,17 +4612,17 @@
       </c>
       <c r="Q81" s="19" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="R81" s="19" t="inlineStr">
         <is>
-          <t>ASM</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S81" s="19" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>WLS</t>
         </is>
       </c>
       <c r="T81" s="19" t="n"/>
@@ -4656,16 +4654,18 @@
       </c>
       <c r="Q82" s="19" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="R82" s="19" t="inlineStr">
         <is>
-          <t>AWP</t>
-        </is>
-      </c>
-      <c r="S82" s="19" t="n">
-        <v/>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="S82" s="19" t="inlineStr">
+        <is>
+          <t>WLS</t>
+        </is>
       </c>
       <c r="T82" s="19" t="n"/>
       <c r="U82" s="19" t="n"/>
@@ -4696,17 +4696,17 @@
       </c>
       <c r="Q83" s="19" t="inlineStr">
         <is>
-          <t>2024-10-15</t>
+          <t>2024-10-21</t>
         </is>
       </c>
       <c r="R83" s="19" t="inlineStr">
         <is>
-          <t>JWA</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S83" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>JHA</t>
         </is>
       </c>
       <c r="T83" s="19" t="n"/>
@@ -4738,7 +4738,7 @@
       </c>
       <c r="Q84" s="19" t="inlineStr">
         <is>
-          <t>2024-10-11</t>
+          <t>2024-10-16</t>
         </is>
       </c>
       <c r="R84" s="19" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="S84" s="19" t="inlineStr">
         <is>
-          <t>LDE</t>
+          <t>CMC</t>
         </is>
       </c>
       <c r="T84" s="19" t="n"/>
@@ -4780,12 +4780,12 @@
       </c>
       <c r="Q85" s="19" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2024-10-16</t>
         </is>
       </c>
       <c r="R85" s="19" t="inlineStr">
         <is>
-          <t>PRT</t>
+          <t>AWP</t>
         </is>
       </c>
       <c r="S85" s="19" t="n">
@@ -4820,16 +4820,18 @@
       </c>
       <c r="Q86" s="19" t="inlineStr">
         <is>
-          <t>2024-10-05</t>
+          <t>2024-10-15</t>
         </is>
       </c>
       <c r="R86" s="19" t="inlineStr">
         <is>
-          <t>PRT</t>
-        </is>
-      </c>
-      <c r="S86" s="19" t="n">
-        <v/>
+          <t>JWA</t>
+        </is>
+      </c>
+      <c r="S86" s="19" t="inlineStr">
+        <is>
+          <t>LDE</t>
+        </is>
       </c>
       <c r="T86" s="19" t="n"/>
       <c r="U86" s="19" t="n"/>
@@ -4860,16 +4862,18 @@
       </c>
       <c r="Q87" s="19" t="inlineStr">
         <is>
-          <t>2024-10-04</t>
+          <t>2024-10-11</t>
         </is>
       </c>
       <c r="R87" s="19" t="inlineStr">
         <is>
-          <t>PRT</t>
-        </is>
-      </c>
-      <c r="S87" s="19" t="n">
-        <v/>
+          <t>ASM</t>
+        </is>
+      </c>
+      <c r="S87" s="19" t="inlineStr">
+        <is>
+          <t>LDE</t>
+        </is>
       </c>
       <c r="T87" s="19" t="n"/>
       <c r="U87" s="19" t="n"/>
@@ -4900,18 +4904,16 @@
       </c>
       <c r="Q88" s="19" t="inlineStr">
         <is>
-          <t>2024-09-26</t>
+          <t>2024-10-05</t>
         </is>
       </c>
       <c r="R88" s="19" t="inlineStr">
         <is>
-          <t>JHA</t>
-        </is>
-      </c>
-      <c r="S88" s="19" t="inlineStr">
-        <is>
-          <t>MIR</t>
-        </is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="S88" s="19" t="n">
+        <v/>
       </c>
       <c r="T88" s="19" t="n"/>
       <c r="U88" s="19" t="n"/>
@@ -4942,12 +4944,12 @@
       </c>
       <c r="Q89" s="19" t="inlineStr">
         <is>
-          <t>2024-09-22</t>
+          <t>2024-10-05</t>
         </is>
       </c>
       <c r="R89" s="19" t="inlineStr">
         <is>
-          <t>TKI</t>
+          <t>PRT</t>
         </is>
       </c>
       <c r="S89" s="19" t="n">
@@ -4982,18 +4984,16 @@
       </c>
       <c r="Q90" s="19" t="inlineStr">
         <is>
-          <t>2024-09-12</t>
+          <t>2024-10-04</t>
         </is>
       </c>
       <c r="R90" s="19" t="inlineStr">
         <is>
-          <t>WSM</t>
-        </is>
-      </c>
-      <c r="S90" s="19" t="inlineStr">
-        <is>
-          <t>WWH</t>
-        </is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="S90" s="19" t="n">
+        <v/>
       </c>
       <c r="T90" s="19" t="n"/>
       <c r="U90" s="19" t="n"/>
@@ -5024,16 +5024,18 @@
       </c>
       <c r="Q91" s="19" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2024-09-26</t>
         </is>
       </c>
       <c r="R91" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
-        </is>
-      </c>
-      <c r="S91" s="19" t="n">
-        <v/>
+          <t>JHA</t>
+        </is>
+      </c>
+      <c r="S91" s="19" t="inlineStr">
+        <is>
+          <t>MIR</t>
+        </is>
       </c>
       <c r="T91" s="19" t="n"/>
       <c r="U91" s="19" t="n"/>
@@ -5064,18 +5066,16 @@
       </c>
       <c r="Q92" s="19" t="inlineStr">
         <is>
-          <t>2024-08-03</t>
+          <t>2024-09-22</t>
         </is>
       </c>
       <c r="R92" s="19" t="inlineStr">
         <is>
-          <t>CSY</t>
-        </is>
-      </c>
-      <c r="S92" s="19" t="inlineStr">
-        <is>
-          <t>PRT</t>
-        </is>
+          <t>TKI</t>
+        </is>
+      </c>
+      <c r="S92" s="19" t="n">
+        <v/>
       </c>
       <c r="T92" s="19" t="n"/>
       <c r="U92" s="19" t="n"/>
@@ -5106,18 +5106,16 @@
       </c>
       <c r="Q93" s="19" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>2024-08-30</t>
         </is>
       </c>
       <c r="R93" s="19" t="inlineStr">
         <is>
-          <t>JPJ</t>
-        </is>
-      </c>
-      <c r="S93" s="19" t="inlineStr">
-        <is>
-          <t>JYK</t>
-        </is>
+          <t>SMB</t>
+        </is>
+      </c>
+      <c r="S93" s="19" t="n">
+        <v/>
       </c>
       <c r="T93" s="19" t="n"/>
       <c r="U93" s="19" t="n"/>
@@ -5148,17 +5146,17 @@
       </c>
       <c r="Q94" s="19" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-08-03</t>
         </is>
       </c>
       <c r="R94" s="19" t="inlineStr">
         <is>
-          <t>MBE</t>
+          <t>CSY</t>
         </is>
       </c>
       <c r="S94" s="19" t="inlineStr">
         <is>
-          <t>RJC</t>
+          <t>PRT</t>
         </is>
       </c>
       <c r="T94" s="19" t="n"/>
@@ -5190,17 +5188,17 @@
       </c>
       <c r="Q95" s="19" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2024-08-02</t>
         </is>
       </c>
       <c r="R95" s="19" t="inlineStr">
         <is>
-          <t>RTH</t>
+          <t>JPJ</t>
         </is>
       </c>
       <c r="S95" s="19" t="inlineStr">
         <is>
-          <t>RUB</t>
+          <t>JYK</t>
         </is>
       </c>
       <c r="T95" s="19" t="n"/>
@@ -5232,16 +5230,18 @@
       </c>
       <c r="Q96" s="19" t="inlineStr">
         <is>
-          <t>2024-06-28</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="R96" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="S96" s="19" t="n">
-        <v/>
+          <t>MBE</t>
+        </is>
+      </c>
+      <c r="S96" s="19" t="inlineStr">
+        <is>
+          <t>RJC</t>
+        </is>
       </c>
       <c r="T96" s="19" t="n"/>
       <c r="U96" s="19" t="n"/>
@@ -5272,16 +5272,18 @@
       </c>
       <c r="Q97" s="19" t="inlineStr">
         <is>
-          <t>2024-06-22</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="R97" s="19" t="inlineStr">
         <is>
-          <t>JPJ</t>
-        </is>
-      </c>
-      <c r="S97" s="19" t="n">
-        <v/>
+          <t>RTH</t>
+        </is>
+      </c>
+      <c r="S97" s="19" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
       </c>
       <c r="T97" s="19" t="n"/>
       <c r="U97" s="19" t="n"/>
@@ -5312,7 +5314,7 @@
       </c>
       <c r="Q98" s="19" t="inlineStr">
         <is>
-          <t>2024-06-15</t>
+          <t>2024-06-28</t>
         </is>
       </c>
       <c r="R98" s="19" t="inlineStr">
@@ -5352,18 +5354,16 @@
       </c>
       <c r="Q99" s="19" t="inlineStr">
         <is>
-          <t>2024-06-14</t>
+          <t>2024-06-22</t>
         </is>
       </c>
       <c r="R99" s="19" t="inlineStr">
         <is>
-          <t>CMC</t>
-        </is>
-      </c>
-      <c r="S99" s="19" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
+          <t>JPJ</t>
+        </is>
+      </c>
+      <c r="S99" s="19" t="n">
+        <v/>
       </c>
       <c r="T99" s="19" t="n"/>
       <c r="U99" s="19" t="n"/>
@@ -5394,12 +5394,12 @@
       </c>
       <c r="Q100" s="19" t="inlineStr">
         <is>
-          <t>2024-05-24</t>
+          <t>2024-06-15</t>
         </is>
       </c>
       <c r="R100" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S100" s="19" t="n">
@@ -5434,16 +5434,18 @@
       </c>
       <c r="Q101" s="19" t="inlineStr">
         <is>
-          <t>2024-05-19</t>
+          <t>2024-06-14</t>
         </is>
       </c>
       <c r="R101" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
-        </is>
-      </c>
-      <c r="S101" s="19" t="n">
-        <v/>
+          <t>CMC</t>
+        </is>
+      </c>
+      <c r="S101" s="19" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
       </c>
       <c r="T101" s="19" t="n"/>
       <c r="U101" s="19" t="n"/>
@@ -5474,12 +5476,12 @@
       </c>
       <c r="Q102" s="19" t="inlineStr">
         <is>
-          <t>2024-05-18</t>
+          <t>2024-05-24</t>
         </is>
       </c>
       <c r="R102" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="S102" s="19" t="n">
@@ -5514,7 +5516,7 @@
       </c>
       <c r="Q103" s="19" t="inlineStr">
         <is>
-          <t>2024-05-17</t>
+          <t>2024-05-19</t>
         </is>
       </c>
       <c r="R103" s="19" t="inlineStr">
@@ -5554,18 +5556,16 @@
       </c>
       <c r="Q104" s="19" t="inlineStr">
         <is>
-          <t>2024-05-17</t>
+          <t>2024-05-18</t>
         </is>
       </c>
       <c r="R104" s="19" t="inlineStr">
         <is>
-          <t>LOV</t>
-        </is>
-      </c>
-      <c r="S104" s="19" t="inlineStr">
-        <is>
-          <t>RTH</t>
-        </is>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="S104" s="19" t="n">
+        <v/>
       </c>
       <c r="T104" s="19" t="n"/>
       <c r="U104" s="19" t="n"/>
@@ -5596,16 +5596,18 @@
       </c>
       <c r="Q105" s="19" t="inlineStr">
         <is>
-          <t>2024-05-07</t>
+          <t>2024-05-17</t>
         </is>
       </c>
       <c r="R105" s="19" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="S105" s="19" t="n">
-        <v/>
+          <t>LOV</t>
+        </is>
+      </c>
+      <c r="S105" s="19" t="inlineStr">
+        <is>
+          <t>RTH</t>
+        </is>
       </c>
       <c r="T105" s="19" t="n"/>
       <c r="U105" s="19" t="n"/>
@@ -5636,12 +5638,12 @@
       </c>
       <c r="Q106" s="19" t="inlineStr">
         <is>
-          <t>2024-04-20</t>
+          <t>2024-05-17</t>
         </is>
       </c>
       <c r="R106" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>DDC</t>
         </is>
       </c>
       <c r="S106" s="19" t="n">
@@ -5676,18 +5678,16 @@
       </c>
       <c r="Q107" s="19" t="inlineStr">
         <is>
-          <t>2024-04-02</t>
+          <t>2024-05-07</t>
         </is>
       </c>
       <c r="R107" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
-        </is>
-      </c>
-      <c r="S107" s="19" t="inlineStr">
-        <is>
-          <t>HMK</t>
-        </is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="S107" s="19" t="n">
+        <v/>
       </c>
       <c r="T107" s="19" t="n"/>
       <c r="U107" s="19" t="n"/>
@@ -5718,12 +5718,12 @@
       </c>
       <c r="Q108" s="19" t="inlineStr">
         <is>
-          <t>2024-03-24</t>
+          <t>2024-04-20</t>
         </is>
       </c>
       <c r="R108" s="19" t="inlineStr">
         <is>
-          <t>PRT</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S108" s="19" t="n">
@@ -5758,16 +5758,18 @@
       </c>
       <c r="Q109" s="19" t="inlineStr">
         <is>
-          <t>2024-03-22</t>
+          <t>2024-04-02</t>
         </is>
       </c>
       <c r="R109" s="19" t="inlineStr">
         <is>
-          <t>PRT</t>
-        </is>
-      </c>
-      <c r="S109" s="19" t="n">
-        <v/>
+          <t>DDC</t>
+        </is>
+      </c>
+      <c r="S109" s="19" t="inlineStr">
+        <is>
+          <t>HMK</t>
+        </is>
       </c>
       <c r="T109" s="19" t="n"/>
       <c r="U109" s="19" t="n"/>
@@ -5798,12 +5800,12 @@
       </c>
       <c r="Q110" s="19" t="inlineStr">
         <is>
-          <t>2024-03-05</t>
+          <t>2024-03-24</t>
         </is>
       </c>
       <c r="R110" s="19" t="inlineStr">
         <is>
-          <t>JPK</t>
+          <t>PRT</t>
         </is>
       </c>
       <c r="S110" s="19" t="n">
@@ -5838,18 +5840,16 @@
       </c>
       <c r="Q111" s="19" t="inlineStr">
         <is>
-          <t>2024-03-03</t>
+          <t>2024-03-22</t>
         </is>
       </c>
       <c r="R111" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="S111" s="19" t="inlineStr">
-        <is>
-          <t>JYK</t>
-        </is>
+          <t>PRT</t>
+        </is>
+      </c>
+      <c r="S111" s="19" t="n">
+        <v/>
       </c>
       <c r="T111" s="19" t="n"/>
       <c r="U111" s="19" t="n"/>
@@ -5880,18 +5880,16 @@
       </c>
       <c r="Q112" s="19" t="inlineStr">
         <is>
-          <t>2024-02-08</t>
+          <t>2024-03-05</t>
         </is>
       </c>
       <c r="R112" s="19" t="inlineStr">
         <is>
-          <t>CSY</t>
-        </is>
-      </c>
-      <c r="S112" s="19" t="inlineStr">
-        <is>
-          <t>PRT</t>
-        </is>
+          <t>JPK</t>
+        </is>
+      </c>
+      <c r="S112" s="19" t="n">
+        <v/>
       </c>
       <c r="T112" s="19" t="n"/>
       <c r="U112" s="19" t="n"/>
@@ -5922,17 +5920,17 @@
       </c>
       <c r="Q113" s="19" t="inlineStr">
         <is>
-          <t>2024-01-26</t>
+          <t>2024-03-03</t>
         </is>
       </c>
       <c r="R113" s="19" t="inlineStr">
         <is>
-          <t>ASM</t>
+          <t>GLO</t>
         </is>
       </c>
       <c r="S113" s="19" t="inlineStr">
         <is>
-          <t>HEI</t>
+          <t>JYK</t>
         </is>
       </c>
       <c r="T113" s="19" t="n"/>
@@ -5964,17 +5962,17 @@
       </c>
       <c r="Q114" s="19" t="inlineStr">
         <is>
-          <t>2023-12-20</t>
+          <t>2024-02-08</t>
         </is>
       </c>
       <c r="R114" s="19" t="inlineStr">
         <is>
-          <t>CMC</t>
+          <t>CSY</t>
         </is>
       </c>
       <c r="S114" s="19" t="inlineStr">
         <is>
-          <t>YAT</t>
+          <t>PRT</t>
         </is>
       </c>
       <c r="T114" s="19" t="n"/>
@@ -6006,17 +6004,17 @@
       </c>
       <c r="Q115" s="19" t="inlineStr">
         <is>
-          <t>2023-11-21</t>
+          <t>2024-01-26</t>
         </is>
       </c>
       <c r="R115" s="19" t="inlineStr">
         <is>
-          <t>JYK</t>
+          <t>ASM</t>
         </is>
       </c>
       <c r="S115" s="19" t="inlineStr">
         <is>
-          <t>WLM</t>
+          <t>HEI</t>
         </is>
       </c>
       <c r="T115" s="19" t="n"/>
@@ -6048,16 +6046,18 @@
       </c>
       <c r="Q116" s="19" t="inlineStr">
         <is>
-          <t>2023-11-20</t>
+          <t>2023-12-20</t>
         </is>
       </c>
       <c r="R116" s="19" t="inlineStr">
         <is>
-          <t>NAY</t>
-        </is>
-      </c>
-      <c r="S116" s="19" t="n">
-        <v/>
+          <t>CMC</t>
+        </is>
+      </c>
+      <c r="S116" s="19" t="inlineStr">
+        <is>
+          <t>YAT</t>
+        </is>
       </c>
       <c r="T116" s="19" t="n"/>
       <c r="U116" s="19" t="n"/>
@@ -6088,12 +6088,12 @@
       </c>
       <c r="Q117" s="19" t="inlineStr">
         <is>
-          <t>2023-11-12</t>
+          <t>2023-11-20</t>
         </is>
       </c>
       <c r="R117" s="19" t="inlineStr">
         <is>
-          <t>DDC</t>
+          <t>NAY</t>
         </is>
       </c>
       <c r="S117" s="19" t="n">
@@ -6168,12 +6168,12 @@
       </c>
       <c r="Q119" s="19" t="inlineStr">
         <is>
-          <t>2023-11-04</t>
+          <t>2023-11-12</t>
         </is>
       </c>
       <c r="R119" s="19" t="inlineStr">
         <is>
-          <t>SMB</t>
+          <t>DDC</t>
         </is>
       </c>
       <c r="S119" s="19" t="n">
@@ -6208,12 +6208,12 @@
       </c>
       <c r="Q120" s="19" t="inlineStr">
         <is>
-          <t>2023-10-08</t>
+          <t>2023-11-04</t>
         </is>
       </c>
       <c r="R120" s="19" t="inlineStr">
         <is>
-          <t>GLO</t>
+          <t>SMB</t>
         </is>
       </c>
       <c r="S120" s="19" t="n">
@@ -6248,18 +6248,16 @@
       </c>
       <c r="Q121" s="19" t="inlineStr">
         <is>
-          <t>2023-10-06</t>
+          <t>2023-10-08</t>
         </is>
       </c>
       <c r="R121" s="19" t="inlineStr">
         <is>
-          <t>TKI</t>
-        </is>
-      </c>
-      <c r="S121" s="19" t="inlineStr">
-        <is>
-          <t>WLS</t>
-        </is>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="S121" s="19" t="n">
+        <v/>
       </c>
       <c r="T121" s="19" t="n"/>
       <c r="U121" s="19" t="n"/>
@@ -6379,12 +6377,12 @@
       </c>
       <c r="R124" s="19" t="inlineStr">
         <is>
-          <t>CWI</t>
+          <t>ASM</t>
         </is>
       </c>
       <c r="S124" s="19" t="inlineStr">
         <is>
-          <t>NAY</t>
+          <t>RJC</t>
         </is>
       </c>
       <c r="T124" s="19" t="n"/>

</xml_diff>